<commit_message>
Build Section 1: cascading LGA/ward/settlement select, enumerator/team lookup, GPS plausibility check, previous-round lookup
</commit_message>
<xml_diff>
--- a/form/HH2026v1.xlsx
+++ b/form/HH2026v1.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026070100</t>
+          <t>2026070200</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,21 +537,36 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>choice_filter</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>readonly</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>begin group</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>form_intro</t>
+          <t>section1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Integrated Child Health and Antimicrobial Resistance Survey 2026 — Household Questionnaire</t>
+          <t>Section 1: Household identification</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -561,6 +576,680 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>select_one lga_list</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>lga</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1.02 Local Government Area</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>select_one_from_file wards.csv</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ward</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1.03 Ward</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>lga_code=${lga}</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>select_one_from_file settlements.csv</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1.04 Settlement</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ward_code=${ward}</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>select_one yesno</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>settlement_known_locally</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1.05 Is the settlement known locally by a different name?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>settlement_local_name</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Name used locally</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>${settlement_known_locally}='1'</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>${settlement_known_locally}='1'</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>structure_number</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1.06 Structure number painted on the dwelling</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 999</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Enter a number between 1 and 999</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>hh_serial_number</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1.07 Household serial number within the settlement</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 999</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Enter a number between 1 and 999</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>select_one_from_file staff_roster.csv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>enumerator_code</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1.08 Enumerator code</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>role='Enumerator'</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>team_code_calc</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>pulldata('staff_roster.csv','team_code','name',${enumerator_code})</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>team_code_display</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1.09 Team code</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>${team_code_calc}</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>visit_date</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1.10 Date of visit</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>. &gt;= date('2026-06-01') and . &lt;= date('2026-06-30')</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Date must be within the fieldwork period, 1-30 June 2026</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>geopoint</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gps_reading</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1.11 Record the GPS reading taken at the entrance to the dwelling.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>gps_lat</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>substring-before(${gps_reading},' ')</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gps_lon</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>substring-before(substring-after(${gps_reading},' '),' ')</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>settlement_lat_calc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>pulldata('settlements.csv','latitude','name',${settlement})</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>settlement_lon_calc</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>pulldata('settlements.csv','longitude','name',${settlement})</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>gps_plausibility_flag</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>This GPS reading looks far from the registered location of the selected settlement. Please confirm this is the correct dwelling before continuing.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>(${gps_reading}!='') and ((abs(number(${gps_lat}) - number(${settlement_lat_calc})) &gt; 0.05) or (abs(number(${gps_lon}) - number(${settlement_lon_calc})) &gt; 0.05))</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>select_one visited_previous_list</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>prev_round_visited</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1.12 Was this household visited during the October 2025 round?</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>prev_household_id</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1.13 Record the household identifier allocated in the October 2025 round.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>${prev_round_visited}='1'</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>pulldata('previous_round_households.csv','household_id','household_id',.) != ''</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>This household ID was not found in the previous round register. Please check and re-enter.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>select_one visit_result_list</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>result_of_visit</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1.14 Result of visit</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -573,7 +1262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,6 +1282,227 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>lga_list</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>LGA02</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gwarin</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lga_list</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>LGA01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Idi-Oro</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>lga_list</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LGA04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ilela</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lga_list</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LGA03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Katsuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>yesno</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>yesno</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>visited_previous_list</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>visited_previous_list</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>visited_previous_list</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Do not know</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>visit_result_list</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>visit_result_list</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>visit_result_list</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>No competent adult after three visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>visit_result_list</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dwelling vacant or demolished</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix pyxform instance-duplication bug (pulldata filename mismatch); log as D03
</commit_message>
<xml_diff>
--- a/form/HH2026v1.xlsx
+++ b/form/HH2026v1.xlsx
@@ -879,7 +879,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>pulldata('staff_roster.csv','team_code','name',${enumerator_code})</t>
+          <t>pulldata('staff_roster','team_code','name',${enumerator_code})</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1065,7 +1065,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>pulldata('settlements.csv','latitude','name',${settlement})</t>
+          <t>pulldata('settlements','latitude','name',${settlement})</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1092,7 +1092,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>pulldata('settlements.csv','longitude','name',${settlement})</t>
+          <t>pulldata('settlements','longitude','name',${settlement})</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>pulldata('previous_round_households.csv','household_id','household_id',.) != ''</t>
+          <t>pulldata('previous_round_households','household_id','household_id',.) != ''</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">

</xml_diff>

<commit_message>
Build Section 4 nested in roster repeat: split sentinel fields, vaccination/antibiotic skip chains, 4.13/4.14 merged per D01
</commit_message>
<xml_diff>
--- a/form/HH2026v1.xlsx
+++ b/form/HH2026v1.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,6 +550,11 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>readonly</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>repeat_count</t>
         </is>
       </c>
     </row>
@@ -579,6 +584,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -610,6 +616,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -645,6 +652,7 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -680,6 +688,7 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -711,6 +720,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -746,6 +756,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -785,6 +796,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -824,6 +836,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -859,6 +872,7 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -886,6 +900,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -921,6 +936,7 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -960,6 +976,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -991,6 +1008,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1018,6 +1036,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1045,6 +1064,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1072,6 +1092,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1099,6 +1120,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1130,6 +1152,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1161,6 +1184,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1200,6 +1224,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1231,6 +1256,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1250,6 +1276,1187 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>section2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Section 2: Consent</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>${result_of_visit}='1'</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>select_one yesno</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>consent_read_aloud</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2.01 Consent statement read aloud to the respondent in full?</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>select_one consent_list</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>consent_given</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2.02 Does the respondent consent to the household interview?</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>select_one relationship_list</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>respondent_relationship</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2.03 Relationship of the respondent to the head of household</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>${consent_given}='1'</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>section3</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Section 3: Household roster</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>${result_of_visit}='1' and ${consent_given}='1'</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>household_size</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>3.01 How many people usually live in this household?</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>. &gt;= 1 and . &lt;= 30</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Enter a number between 1 and 30</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>begin repeat</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>roster</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Household roster</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>${household_size}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>name_initials</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>(2) Name or initials</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>select_one relationship_list</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>relationship_to_head</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>(3) Relationship to head</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>select_one sex_list</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>(4) Sex</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>select_one yesno</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>under5</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Is this person under 5 years old?</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>age_years</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>(5) Age in completed years</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>${under5}='2'</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>${under5}='2'</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>. &gt;= 5 and . &lt;= 120</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Enter age in completed years, 5 or older</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>age_months</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>(6) Age in completed months (under 5 only)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>${under5}='1'</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>${under5}='1'</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 59</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Enter age in completed months, 0 to 59</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>eligible_for_section4</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>if(${under5}='1' and ${age_months} &gt;= 9 and ${age_months} &lt;= 59, 1, 0)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>section4_module</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Section 4: Child module</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>${eligible_for_section4}='1'</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>roster_line_number</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>position(..)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>s4_child_ref</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>This module is for: ${name_initials}, ${age_months} months, line ${roster_line_number}</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>select_one measured_status_list</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>weight_status</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>4.05 Weight of the child</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>weight_kg</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Weight (kg)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>${weight_status}='1'</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>${weight_status}='1'</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>. &gt;= 2.0 and . &lt;= 30.0</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Enter weight in kg, 2.0 to 30.0</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>select_one measured_status_list</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>height_status</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>4.06 Length or height of the child</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>height_cm</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Length or height (cm)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>${height_status}='1'</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>${height_status}='1'</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>. &gt;= 60.0 and . &lt;= 120.0</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Enter length/height in cm, 60.0 to 120.0</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>select_one position_list</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>measurement_position</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>4.07 Position in which the child was measured</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>${height_status}='1'</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>${height_status}='1'</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>select_one card_seen_list</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>card_seen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>4.08 May I see the child's vaccination card or health record?</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>select_one yesno</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>measles_on_card</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>4.09 Copy from the card: is a measles dose recorded?</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>${card_seen}='1'</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>${card_seen}='1'</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>select_one yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>measles_ever</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>4.10 Has this child ever received a measles vaccination?</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>${card_seen}='2'</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>${card_seen}='2'</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>select_one yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>diarrhoea_14d</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>4.11 Has this child had diarrhoea in the past 14 days?</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>select_one yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>antibiotic_30d</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>4.12 Has this child taken any antibiotic medicine in the past 30 days?</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>antibiotic_name</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>4.13/4.14 Which antibiotic was taken? Record the name as reported by the caregiver.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>OPEN ITEM: no controlled medicine list was supplied with the data pack (see defects log D01). Recorded as free text pending that list.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>${antibiotic_30d}='1'</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>${antibiotic_30d}='1'</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>select_one yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>antibiotic_no_prescription</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>4.15 Was the medicine obtained without a prescription from a health worker?</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>${antibiotic_30d}='1'</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>${antibiotic_30d}='1'</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>select_one photo_taken_list</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>antibiotic_photo_taken</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>4.16 Was a photograph of the medicine packaging taken?</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>${antibiotic_30d}='1'</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>${antibiotic_30d}='1'</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>end repeat</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>eligible_children_count</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>sum(../roster/eligible_for_section4)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>eligible_children_display</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>3.02 Number of children aged 9 to 59 completed months (calculated automatically from the roster)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>${eligible_children_count}</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1262,7 +2469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1503,6 +2710,380 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>consent_list</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Consent given</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>consent_list</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Consent refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>relationship_list</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>relationship_list</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Spouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>relationship_list</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Son or daughter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>relationship_list</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>relationship_list</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Other relative</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>relationship_list</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Not related</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sex_list</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sex_list</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Do not know</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>measured_status_list</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>measured_status_list</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Not measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>card_seen_list</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Card seen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>card_seen_list</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>No card seen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>position_list</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Recumbent length</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>position_list</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Standing height</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>photo_taken_list</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>photo_taken_list</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>No, not available</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>photo_taken_list</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Caregiver declined</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Build Section 5: specimen check-digit logic hand-unrolled in XPath, verified against reference script on both test cases
</commit_message>
<xml_diff>
--- a/form/HH2026v1.xlsx
+++ b/form/HH2026v1.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2357,14 +2357,26 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>end repeat</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>section5_module</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Section 5: Specimen collection</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>${eligible_for_section4}='1'</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
@@ -2377,25 +2389,29 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>select_one yesno</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>eligible_children_count</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr"/>
+          <t>age12plus</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>5.01 Is the child aged 12 completed months or older?</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>sum(../roster/eligible_for_section4)</t>
-        </is>
-      </c>
+      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
@@ -2405,58 +2421,710 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one yesno</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>eligible_children_display</t>
+          <t>specimen_obtained</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>3.02 Number of children aged 9 to 59 completed months (calculated automatically from the roster)</t>
+          <t>5.02 Was a stool specimen obtained from this child?</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>${age12plus}='1'</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>${age12plus}='1'</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>${eligible_children_count}</t>
-        </is>
-      </c>
+      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>end group</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>specimen_number</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>5.03 Specimen label number (6 digits printed after the BSN prefix)</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>regex(.,'^[0-9]{6}$') and number(.) &gt;= number(${range_start_calc}) and number(.) &lt;= number(${range_end_calc})</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Must be exactly 6 digits and within your team's issued label range (${range_start_calc}-${range_end_calc})</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>range_start_calc</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>pulldata('specimen_label_allocation','range_start','team_code',${team_code_calc})</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>range_end_calc</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>pulldata('specimen_label_allocation','range_end','team_code',${team_code_calc})</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>specimen_digit0</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>if(string-length(${specimen_number})=6, number(substr(${specimen_number},0,1)), 0)</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>specimen_digit1</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>if(string-length(${specimen_number})=6, number(substr(${specimen_number},1,2)), 0)</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>specimen_digit2</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>if(string-length(${specimen_number})=6, number(substr(${specimen_number},2,3)), 0)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>specimen_digit3</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>if(string-length(${specimen_number})=6, number(substr(${specimen_number},3,4)), 0)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>specimen_digit4</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>if(string-length(${specimen_number})=6, number(substr(${specimen_number},4,5)), 0)</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>specimen_digit5</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>if(string-length(${specimen_number})=6, number(substr(${specimen_number},5,6)), 0)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>specimen_weighted_sum</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>(${specimen_digit0}*7)+(${specimen_digit1}*6)+(${specimen_digit2}*5)+(${specimen_digit3}*4)+(${specimen_digit4}*3)+(${specimen_digit5}*2)</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>specimen_remainder</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>${specimen_weighted_sum} mod 11</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>specimen_computed_check_digit</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>if(${specimen_remainder}=0,'0',if(${specimen_remainder}=1,'X',string(11 - ${specimen_remainder})))</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>specimen_check_digit</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Check digit (single digit 0-9, or X)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>. = ${specimen_computed_check_digit}</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Check digit does not match this label number. Please re-check both and re-enter.</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>specimen_coldbox_time</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>5.04 Time the specimen was placed in the cold box</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>specimen_coldbox_temp</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>5.05 Temperature shown on the cold box thermometer at that time</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='1'</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>. &gt;= 2.0 and . &lt;= 8.0</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Enter a temperature between 2.0 and 8.0 degrees C</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>select_one reason_no_specimen_list</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>reason_no_specimen</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>5.06 Reason no specimen was obtained</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='2'</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>${specimen_obtained}='2'</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>reason_no_specimen_other</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>5.07 If code 96, specify</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>${reason_no_specimen}='96'</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>${reason_no_specimen}='96'</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>end repeat</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>eligible_children_count</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>sum(../roster/eligible_for_section4)</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>eligible_children_display</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>3.02 Number of children aged 9 to 59 completed months (calculated automatically from the roster)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>${eligible_children_count}</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2469,7 +3137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3084,6 +3752,91 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>reason_no_specimen_list</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Caregiver refused</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>reason_no_specimen_list</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Child absent</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>reason_no_specimen_list</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Unable to produce</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>reason_no_specimen_list</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Container spoiled</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>reason_no_specimen_list</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Build Sections 6-7: household environment, asset ownership with mutual-exclusion constraint, supervisor close-out. All 7 sections complete.
</commit_message>
<xml_diff>
--- a/form/HH2026v1.xlsx
+++ b/form/HH2026v1.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3126,6 +3126,602 @@
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>section6</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Section 6: Household environment</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>${result_of_visit}='1' and ${consent_given}='1'</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>select_one water_source_list</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>water_source</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>6.01 What is the main source of drinking water for members of this household?</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>select_one toilet_list</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>toilet_type</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>6.02 What kind of toilet facility do members of this household usually use?</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>select_one yesno</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>keeps_animals</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>6.03 Does this household keep poultry or livestock inside the compound?</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>select_one yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>animal_antibiotics_12m</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>6.04 Have any antibiotic medicines been given to these animals in the past 12 months?</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>${keeps_animals}='1'</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>${keeps_animals}='1'</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>select_one handwashing_list</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>handwashing_station</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>6.05 Observe: is there a handwashing station with both soap and water available?</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>select_one yesnodk_list</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>hh_diarrhoea_2w</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>6.06 Has any member of this household had diarrhoea in the past two weeks?</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>select_multiple assets_list</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>household_assets</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>6.07 Which of the following does this household own?</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>not(selected(., 'H')) or count-selected(.) = 1</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>'None of these' cannot be selected together with any other option</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>begin group</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>section7</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Section 7: Close-out and supervisor review</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>${result_of_visit}='1' and ${consent_given}='1'</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>interview_end_time</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>7.01 Time the interview ended</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>office_observation</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>7.02 Record any observation that may help the office interpret this form.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>enumerator_signature</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>7.03 Enumerator signature</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>enumerator_signature_date</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Enumerator signature date</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>select_one_from_file staff_roster.csv</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>supervisor_code</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>7.04 Supervisor code</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>role='Supervisor'</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>select_one supervisor_decision_list</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>supervisor_decision</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>7.05 Supervisor decision on this form</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>supervisor_signature</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>7.06 Supervisor signature</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>supervisor_signature_date</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Supervisor signature date</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>end group</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3137,7 +3733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3837,6 +4433,584 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Piped into dwelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Piped into compound</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Public tap or standpipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Tube well or borehole</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Protected dug well</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Unprotected dug well</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Protected spring</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Unprotected spring</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Rainwater</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Tanker or cart</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>water_source_list</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Surface water</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Flush to sewer</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Flush to septic tank</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Flush to pit latrine</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Ventilated improved pit</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Pit latrine with slab</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Pit latrine without slab</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Composting toilet</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Bucket</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>toilet_list</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>No facility or bush</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>handwashing_list</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Observed, soap and water</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>handwashing_list</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Reported only, not observed</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>handwashing_list</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Not present</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Television</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Mobile telephone</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Bicycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Motorcycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Car or truck</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Refrigerator</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>assets_list</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>None of these</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>supervisor_decision_list</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>supervisor_decision_list</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Return for correction</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>supervisor_decision_list</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Void</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>